<commit_message>
fix: add SO/BB/HR to pitcher 140-game scaling cols
</commit_message>
<xml_diff>
--- a/ottoneu_power_rankings.xlsx
+++ b/ottoneu_power_rankings.xlsx
@@ -655,13 +655,13 @@
         <v>44.1</v>
       </c>
       <c r="S2" t="n">
-        <v>1771.8</v>
+        <v>1531.2</v>
       </c>
       <c r="T2" t="n">
-        <v>572.7</v>
+        <v>494.9</v>
       </c>
       <c r="U2" t="n">
-        <v>207.1</v>
+        <v>179</v>
       </c>
       <c r="V2" t="n">
         <v>3.75</v>
@@ -764,13 +764,13 @@
         <v>57.8</v>
       </c>
       <c r="S3" t="n">
-        <v>1831</v>
+        <v>1582.4</v>
       </c>
       <c r="T3" t="n">
-        <v>541.9</v>
+        <v>468.3</v>
       </c>
       <c r="U3" t="n">
-        <v>192.3</v>
+        <v>166.2</v>
       </c>
       <c r="V3" t="n">
         <v>3.51</v>
@@ -873,13 +873,13 @@
         <v>23.3</v>
       </c>
       <c r="S4" t="n">
-        <v>1813.4</v>
+        <v>1567.2</v>
       </c>
       <c r="T4" t="n">
-        <v>501.1</v>
+        <v>433</v>
       </c>
       <c r="U4" t="n">
-        <v>187.8</v>
+        <v>162.3</v>
       </c>
       <c r="V4" t="n">
         <v>3.43</v>
@@ -982,13 +982,13 @@
         <v>48.4</v>
       </c>
       <c r="S5" t="n">
-        <v>1819.1</v>
+        <v>1572</v>
       </c>
       <c r="T5" t="n">
-        <v>564.1</v>
+        <v>487.5</v>
       </c>
       <c r="U5" t="n">
-        <v>199.2</v>
+        <v>172.2</v>
       </c>
       <c r="V5" t="n">
         <v>3.64</v>
@@ -1091,13 +1091,13 @@
         <v>55.3</v>
       </c>
       <c r="S6" t="n">
-        <v>1798.5</v>
+        <v>1554.3</v>
       </c>
       <c r="T6" t="n">
-        <v>567.5</v>
+        <v>490.4</v>
       </c>
       <c r="U6" t="n">
-        <v>218</v>
+        <v>188.4</v>
       </c>
       <c r="V6" t="n">
         <v>3.79</v>
@@ -1200,13 +1200,13 @@
         <v>30.2</v>
       </c>
       <c r="S7" t="n">
-        <v>1730</v>
+        <v>1495.1</v>
       </c>
       <c r="T7" t="n">
-        <v>569.7</v>
+        <v>492.3</v>
       </c>
       <c r="U7" t="n">
-        <v>196.8</v>
+        <v>170.1</v>
       </c>
       <c r="V7" t="n">
         <v>3.73</v>
@@ -1309,13 +1309,13 @@
         <v>45.8</v>
       </c>
       <c r="S8" t="n">
-        <v>1681.6</v>
+        <v>1453.2</v>
       </c>
       <c r="T8" t="n">
-        <v>533.5</v>
+        <v>461.1</v>
       </c>
       <c r="U8" t="n">
-        <v>195.8</v>
+        <v>169.2</v>
       </c>
       <c r="V8" t="n">
         <v>3.74</v>
@@ -1418,13 +1418,13 @@
         <v>47.4</v>
       </c>
       <c r="S9" t="n">
-        <v>1708.1</v>
+        <v>1476.2</v>
       </c>
       <c r="T9" t="n">
-        <v>586</v>
+        <v>506.5</v>
       </c>
       <c r="U9" t="n">
-        <v>203.5</v>
+        <v>175.9</v>
       </c>
       <c r="V9" t="n">
         <v>3.91</v>
@@ -1527,13 +1527,13 @@
         <v>34.8</v>
       </c>
       <c r="S10" t="n">
-        <v>1675.6</v>
+        <v>1448</v>
       </c>
       <c r="T10" t="n">
-        <v>606.4</v>
+        <v>524</v>
       </c>
       <c r="U10" t="n">
-        <v>179.2</v>
+        <v>154.8</v>
       </c>
       <c r="V10" t="n">
         <v>3.77</v>
@@ -1636,13 +1636,13 @@
         <v>44.1</v>
       </c>
       <c r="S11" t="n">
-        <v>1566</v>
+        <v>1353.3</v>
       </c>
       <c r="T11" t="n">
-        <v>501</v>
+        <v>433</v>
       </c>
       <c r="U11" t="n">
-        <v>184</v>
+        <v>159</v>
       </c>
       <c r="V11" t="n">
         <v>3.77</v>
@@ -1745,13 +1745,13 @@
         <v>71.5</v>
       </c>
       <c r="S12" t="n">
-        <v>1351.6</v>
+        <v>1168</v>
       </c>
       <c r="T12" t="n">
-        <v>467.1</v>
+        <v>403.7</v>
       </c>
       <c r="U12" t="n">
-        <v>176.6</v>
+        <v>152.6</v>
       </c>
       <c r="V12" t="n">
         <v>3.93</v>
@@ -1854,13 +1854,13 @@
         <v>51.6</v>
       </c>
       <c r="S13" t="n">
-        <v>1625</v>
+        <v>1404.3</v>
       </c>
       <c r="T13" t="n">
-        <v>566.4</v>
+        <v>489.4</v>
       </c>
       <c r="U13" t="n">
-        <v>179.1</v>
+        <v>154.8</v>
       </c>
       <c r="V13" t="n">
         <v>3.78</v>

</xml_diff>